<commit_message>
docs: update Assessment 1 submission workbook with video URL
</commit_message>
<xml_diff>
--- a/Assessment1_Nataraj_Chandrasekaran.xlsx
+++ b/Assessment1_Nataraj_Chandrasekaran.xlsx
@@ -827,7 +827,7 @@
       </c>
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>PSG College of Technology, Coimbatore — B.E. Electronics and Communication Engineering</t>
+          <t>PSG College of Technology, Coimbatore - B.E. Electronics and Communication Engineering</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>https://youtu.be/incubrix_ps1_demo</t>
+          <t>https://youtu.be/cS9gKA6OBIU</t>
         </is>
       </c>
     </row>

</xml_diff>